<commit_message>
Verifica settimanale: doppio controllo AI su 15 file Malesia (124 upgrade)
Doppio controllo indipendente via WebSearch (9 agenti paralleli) sulle
136 righe "DA VERIFICARE UMANAMENTE" nei 15 file nuovi (Malesia, Johor/
Kedah/Kelantan): 124 righe promosse a "VERIFICATA AI - doppio controllo
(01/10/2026)" con conferma reale e coerenza di settore; 12 lasciate
invariate per esito non confermato o settore incoerente (vedi dettaglio
in weekly_verify_log.md). Nessuna riga declassata, nessuna conferma
inventata. Aggiornati weekly_verify_state.json e weekly_verify_log.md.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V1d3BH14wLEVTJJVMB11Ey
</commit_message>
<xml_diff>
--- a/output/2026-09-30_16_Malesia_Johor_Cleaning.xlsx
+++ b/output/2026-09-30_16_Malesia_Johor_Cleaning.xlsx
@@ -506,7 +506,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (01/10/2026)</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (01/10/2026)</t>
         </is>
       </c>
     </row>
@@ -590,7 +590,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (01/10/2026)</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (01/10/2026)</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (01/10/2026)</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (01/10/2026)</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (01/10/2026)</t>
         </is>
       </c>
     </row>
@@ -800,7 +800,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (01/10/2026)</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,6 @@
           <t>+60-149372872</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>Verificato via WebFetch+WebSearch: pagine dedicate a 'Dust Collector Air Purifying System' e 'Fume Extractor' confermate sul sito ufficiale. Azienda generalista (laser cutting, automazione) ma con offerta specifica e verificabile nel settore cleaning/filtrazione aria - incluso con nota di marginalità. Email non reperita su fonti verificate, lasciata vuota.</t>
@@ -838,7 +837,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (01/10/2026)</t>
         </is>
       </c>
     </row>
@@ -880,7 +879,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (01/10/2026)</t>
         </is>
       </c>
     </row>
@@ -922,7 +921,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (01/10/2026)</t>
         </is>
       </c>
     </row>
@@ -964,7 +963,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (01/10/2026)</t>
         </is>
       </c>
     </row>
@@ -1006,7 +1005,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (01/10/2026)</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1047,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (01/10/2026)</t>
         </is>
       </c>
     </row>
@@ -1090,7 +1089,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (01/10/2026)</t>
         </is>
       </c>
     </row>

</xml_diff>